<commit_message>
Update test case files and database for integration login tests
</commit_message>
<xml_diff>
--- a/TestCase_Integration_login.xlsx
+++ b/TestCase_Integration_login.xlsx
@@ -8,22 +8,20 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Desktop\travel_auto_test\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A420A77D-D735-49CB-AFB2-8557B3E36D1F}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2DF6685-BBD8-49D9-9E68-B32101252804}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="480" yWindow="60" windowWidth="18192" windowHeight="8508" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView minimized="1" xWindow="480" yWindow="60" windowWidth="18192" windowHeight="8508" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
-    <sheet name="login" sheetId="2" r:id="rId2"/>
-    <sheet name="search" sheetId="5" r:id="rId3"/>
-    <sheet name="Sheet3" sheetId="4" r:id="rId4"/>
+    <sheet name="login" sheetId="2" r:id="rId1"/>
+    <sheet name="search" sheetId="5" r:id="rId2"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="199" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="62">
   <si>
     <t>Test Case ID</t>
   </si>
@@ -178,74 +176,49 @@
 password = "Hoang"</t>
   </si>
   <si>
-    <t>integration test charge and checkout no discount</t>
-  </si>
-  <si>
-    <t xml:space="preserve">balance = 100
-order_id = 1
-amount = 20
-discount = 0
-</t>
-  </si>
-  <si>
-    <t>checkout return True
-balance = 80
-status = "PAID"</t>
-  </si>
-  <si>
-    <t>integration test charge and checkout with discount</t>
-  </si>
-  <si>
-    <t xml:space="preserve">balance = 100
-order_id = 2
-amount = 50
-discount = 0.2
-</t>
-  </si>
-  <si>
-    <t>checkout return True
-balance = 60
-status = "PAID"</t>
-  </si>
-  <si>
-    <t>integration test charge and checkout with discount and small amount</t>
-  </si>
-  <si>
-    <t xml:space="preserve">balance = 100
-order_id = 3
-amount = 0.5
-discount = 0.5
-</t>
-  </si>
-  <si>
-    <t>checkout return True
-balance = 99.75
-status = "PAID"</t>
-  </si>
-  <si>
-    <t>integration test charge and checkout with not enough balance</t>
-  </si>
-  <si>
-    <t xml:space="preserve">balance = 100
-order_id = 4
-amount = 150
-discount = 0.1
-</t>
-  </si>
-  <si>
-    <t>checkout return False
-balance = 100
-status = "NEW"</t>
-  </si>
-  <si>
-    <t>integration test charge and checkout with invalid discount value</t>
-  </si>
-  <si>
-    <t xml:space="preserve">balance = 100
-order_id = 5
-amount = 50
-discount = 1.5
-</t>
+    <t>A trip to New York shows up</t>
+  </si>
+  <si>
+    <t>Search flight</t>
+  </si>
+  <si>
+    <t>navigate to services, enter flight</t>
+  </si>
+  <si>
+    <t>Search hotel</t>
+  </si>
+  <si>
+    <t>Search hotel but uppercase destination</t>
+  </si>
+  <si>
+    <t>navigate to services, enter hotel</t>
+  </si>
+  <si>
+    <t>hotel = "New york"
+Flight = ""</t>
+  </si>
+  <si>
+    <t>hotel = ""
+Flight = "A380"</t>
+  </si>
+  <si>
+    <t>hotel = "NEW YORK"
+Flight = ""</t>
+  </si>
+  <si>
+    <t>at least one hotel named New York</t>
+  </si>
+  <si>
+    <t>at least one flight named A380</t>
+  </si>
+  <si>
+    <t>Search flight but lowercase flight</t>
+  </si>
+  <si>
+    <t>Found a trip to New York</t>
+  </si>
+  <si>
+    <t>navigate to services, enter hotel name, press button search</t>
   </si>
 </sst>
 </file>
@@ -322,7 +295,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -350,9 +323,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -655,551 +625,6 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <sheetPr>
-    <outlinePr summaryBelow="0"/>
-  </sheetPr>
-  <dimension ref="A1:Q23"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="13.5546875" style="10" hidden="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="20.6640625" style="10" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.5546875" style="10" hidden="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="35.6640625" style="10" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.5546875" style="10" hidden="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="43.6640625" style="10" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13.5546875" style="10" hidden="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="19.33203125" style="10" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="15.6640625" style="10" bestFit="1" customWidth="1"/>
-    <col min="10" max="16" width="13.5546875" style="10" hidden="1" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="13.5546875" style="10" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:17" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="J1" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="K1" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="L1" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="M1" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="N1" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="O1" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="P1" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="Q1" s="5"/>
-    </row>
-    <row r="2" spans="1:17" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="5"/>
-      <c r="B2" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="C2" s="5"/>
-      <c r="D2" s="5" t="s">
-        <v>48</v>
-      </c>
-      <c r="E2" s="5"/>
-      <c r="F2" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="G2" s="5"/>
-      <c r="H2" s="5" t="s">
-        <v>50</v>
-      </c>
-      <c r="I2" s="5" t="s">
-        <v>50</v>
-      </c>
-      <c r="J2" s="5"/>
-      <c r="K2" s="5"/>
-      <c r="L2" s="5"/>
-      <c r="M2" s="5"/>
-      <c r="N2" s="5"/>
-      <c r="O2" s="5"/>
-      <c r="P2" s="5"/>
-      <c r="Q2" s="5"/>
-    </row>
-    <row r="3" spans="1:17" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="5"/>
-      <c r="B3" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="C3" s="5"/>
-      <c r="D3" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="E3" s="5"/>
-      <c r="F3" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="G3" s="5"/>
-      <c r="H3" s="5" t="s">
-        <v>53</v>
-      </c>
-      <c r="I3" s="5" t="s">
-        <v>53</v>
-      </c>
-      <c r="J3" s="5"/>
-      <c r="K3" s="5"/>
-      <c r="L3" s="5"/>
-      <c r="M3" s="5"/>
-      <c r="N3" s="5"/>
-      <c r="O3" s="5"/>
-      <c r="P3" s="5"/>
-      <c r="Q3" s="5"/>
-    </row>
-    <row r="4" spans="1:17" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="5"/>
-      <c r="B4" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="C4" s="5"/>
-      <c r="D4" s="5" t="s">
-        <v>54</v>
-      </c>
-      <c r="E4" s="5"/>
-      <c r="F4" s="5" t="s">
-        <v>55</v>
-      </c>
-      <c r="G4" s="5"/>
-      <c r="H4" s="5" t="s">
-        <v>56</v>
-      </c>
-      <c r="I4" s="5" t="s">
-        <v>56</v>
-      </c>
-      <c r="J4" s="5"/>
-      <c r="K4" s="5"/>
-      <c r="L4" s="5"/>
-      <c r="M4" s="5"/>
-      <c r="N4" s="5"/>
-      <c r="O4" s="5"/>
-      <c r="P4" s="5"/>
-      <c r="Q4" s="5"/>
-    </row>
-    <row r="5" spans="1:17" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="5"/>
-      <c r="B5" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="C5" s="5"/>
-      <c r="D5" s="5" t="s">
-        <v>57</v>
-      </c>
-      <c r="E5" s="5"/>
-      <c r="F5" s="5" t="s">
-        <v>58</v>
-      </c>
-      <c r="G5" s="5"/>
-      <c r="H5" s="5" t="s">
-        <v>59</v>
-      </c>
-      <c r="I5" s="5" t="s">
-        <v>59</v>
-      </c>
-      <c r="J5" s="5"/>
-      <c r="K5" s="5"/>
-      <c r="L5" s="5"/>
-      <c r="M5" s="5"/>
-      <c r="N5" s="5"/>
-      <c r="O5" s="5"/>
-      <c r="P5" s="5"/>
-      <c r="Q5" s="5"/>
-    </row>
-    <row r="6" spans="1:17" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="5"/>
-      <c r="B6" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="C6" s="5"/>
-      <c r="D6" s="5" t="s">
-        <v>60</v>
-      </c>
-      <c r="E6" s="5"/>
-      <c r="F6" s="5" t="s">
-        <v>61</v>
-      </c>
-      <c r="G6" s="5"/>
-      <c r="H6" s="5" t="s">
-        <v>59</v>
-      </c>
-      <c r="I6" s="5" t="s">
-        <v>59</v>
-      </c>
-      <c r="J6" s="5"/>
-      <c r="K6" s="5"/>
-      <c r="L6" s="5"/>
-      <c r="M6" s="5"/>
-      <c r="N6" s="5"/>
-      <c r="O6" s="5"/>
-      <c r="P6" s="5"/>
-      <c r="Q6" s="5"/>
-    </row>
-    <row r="7" spans="1:17" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="5"/>
-      <c r="B7" s="5"/>
-      <c r="C7" s="5"/>
-      <c r="D7" s="5"/>
-      <c r="E7" s="5"/>
-      <c r="F7" s="5"/>
-      <c r="G7" s="5"/>
-      <c r="H7" s="5"/>
-      <c r="I7" s="5"/>
-      <c r="J7" s="5"/>
-      <c r="K7" s="5"/>
-      <c r="L7" s="5"/>
-      <c r="M7" s="5"/>
-      <c r="N7" s="5"/>
-      <c r="O7" s="5"/>
-      <c r="P7" s="5"/>
-      <c r="Q7" s="5"/>
-    </row>
-    <row r="8" spans="1:17" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="5"/>
-      <c r="B8" s="5"/>
-      <c r="C8" s="5"/>
-      <c r="D8" s="5"/>
-      <c r="E8" s="5"/>
-      <c r="F8" s="5"/>
-      <c r="G8" s="5"/>
-      <c r="H8" s="5"/>
-      <c r="I8" s="5"/>
-      <c r="J8" s="5"/>
-      <c r="K8" s="5"/>
-      <c r="L8" s="5"/>
-      <c r="M8" s="5"/>
-      <c r="N8" s="5"/>
-      <c r="O8" s="5"/>
-      <c r="P8" s="5"/>
-      <c r="Q8" s="5"/>
-    </row>
-    <row r="9" spans="1:17" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="5"/>
-      <c r="B9" s="5"/>
-      <c r="C9" s="5"/>
-      <c r="D9" s="5"/>
-      <c r="E9" s="5"/>
-      <c r="F9" s="5"/>
-      <c r="G9" s="5"/>
-      <c r="H9" s="5"/>
-      <c r="I9" s="5"/>
-      <c r="J9" s="5"/>
-      <c r="K9" s="5"/>
-      <c r="L9" s="5"/>
-      <c r="M9" s="5"/>
-      <c r="N9" s="5"/>
-      <c r="O9" s="5"/>
-      <c r="P9" s="5"/>
-      <c r="Q9" s="5"/>
-    </row>
-    <row r="10" spans="1:17" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="5"/>
-      <c r="B10" s="5"/>
-      <c r="C10" s="5"/>
-      <c r="D10" s="5"/>
-      <c r="E10" s="5"/>
-      <c r="F10" s="5"/>
-      <c r="G10" s="5"/>
-      <c r="H10" s="5"/>
-      <c r="I10" s="5"/>
-      <c r="J10" s="5"/>
-      <c r="K10" s="5"/>
-      <c r="L10" s="5"/>
-      <c r="M10" s="5"/>
-      <c r="N10" s="5"/>
-      <c r="O10" s="5"/>
-      <c r="P10" s="5"/>
-      <c r="Q10" s="5"/>
-    </row>
-    <row r="11" spans="1:17" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="5"/>
-      <c r="B11" s="5"/>
-      <c r="C11" s="5"/>
-      <c r="D11" s="5"/>
-      <c r="E11" s="5"/>
-      <c r="F11" s="5"/>
-      <c r="G11" s="5"/>
-      <c r="H11" s="5"/>
-      <c r="I11" s="5"/>
-      <c r="J11" s="5"/>
-      <c r="K11" s="5"/>
-      <c r="L11" s="5"/>
-      <c r="M11" s="5"/>
-      <c r="N11" s="5"/>
-      <c r="O11" s="5"/>
-      <c r="P11" s="5"/>
-      <c r="Q11" s="5"/>
-    </row>
-    <row r="12" spans="1:17" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="5"/>
-      <c r="B12" s="5"/>
-      <c r="C12" s="5"/>
-      <c r="D12" s="5"/>
-      <c r="E12" s="5"/>
-      <c r="F12" s="5"/>
-      <c r="G12" s="5"/>
-      <c r="H12" s="5"/>
-      <c r="I12" s="5"/>
-      <c r="J12" s="5"/>
-      <c r="K12" s="5"/>
-      <c r="L12" s="5"/>
-      <c r="M12" s="5"/>
-      <c r="N12" s="5"/>
-      <c r="O12" s="5"/>
-      <c r="P12" s="5"/>
-      <c r="Q12" s="5"/>
-    </row>
-    <row r="13" spans="1:17" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="5"/>
-      <c r="B13" s="5"/>
-      <c r="C13" s="5"/>
-      <c r="D13" s="5"/>
-      <c r="E13" s="5"/>
-      <c r="F13" s="5"/>
-      <c r="G13" s="5"/>
-      <c r="H13" s="5"/>
-      <c r="I13" s="5"/>
-      <c r="J13" s="5"/>
-      <c r="K13" s="5"/>
-      <c r="L13" s="5"/>
-      <c r="M13" s="5"/>
-      <c r="N13" s="5"/>
-      <c r="O13" s="5"/>
-      <c r="P13" s="5"/>
-      <c r="Q13" s="5"/>
-    </row>
-    <row r="14" spans="1:17" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="5"/>
-      <c r="B14" s="5"/>
-      <c r="C14" s="5"/>
-      <c r="D14" s="5"/>
-      <c r="E14" s="5"/>
-      <c r="F14" s="5"/>
-      <c r="G14" s="5"/>
-      <c r="H14" s="5"/>
-      <c r="I14" s="5"/>
-      <c r="J14" s="5"/>
-      <c r="K14" s="5"/>
-      <c r="L14" s="5"/>
-      <c r="M14" s="5"/>
-      <c r="N14" s="5"/>
-      <c r="O14" s="5"/>
-      <c r="P14" s="5"/>
-      <c r="Q14" s="5"/>
-    </row>
-    <row r="15" spans="1:17" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="5"/>
-      <c r="B15" s="5"/>
-      <c r="C15" s="5"/>
-      <c r="D15" s="5"/>
-      <c r="E15" s="5"/>
-      <c r="F15" s="5"/>
-      <c r="G15" s="5"/>
-      <c r="H15" s="5"/>
-      <c r="I15" s="5"/>
-      <c r="J15" s="5"/>
-      <c r="K15" s="5"/>
-      <c r="L15" s="5"/>
-      <c r="M15" s="5"/>
-      <c r="N15" s="5"/>
-      <c r="O15" s="5"/>
-      <c r="P15" s="5"/>
-      <c r="Q15" s="5"/>
-    </row>
-    <row r="16" spans="1:17" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="5"/>
-      <c r="B16" s="5"/>
-      <c r="C16" s="5"/>
-      <c r="D16" s="5"/>
-      <c r="E16" s="5"/>
-      <c r="F16" s="5"/>
-      <c r="G16" s="5"/>
-      <c r="H16" s="5"/>
-      <c r="I16" s="5"/>
-      <c r="J16" s="5"/>
-      <c r="K16" s="5"/>
-      <c r="L16" s="5"/>
-      <c r="M16" s="5"/>
-      <c r="N16" s="5"/>
-      <c r="O16" s="5"/>
-      <c r="P16" s="5"/>
-      <c r="Q16" s="5"/>
-    </row>
-    <row r="17" spans="1:17" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="5"/>
-      <c r="B17" s="5"/>
-      <c r="C17" s="5"/>
-      <c r="D17" s="5"/>
-      <c r="E17" s="5"/>
-      <c r="F17" s="5"/>
-      <c r="G17" s="5"/>
-      <c r="H17" s="5"/>
-      <c r="I17" s="5"/>
-      <c r="J17" s="5"/>
-      <c r="K17" s="5"/>
-      <c r="L17" s="5"/>
-      <c r="M17" s="5"/>
-      <c r="N17" s="5"/>
-      <c r="O17" s="5"/>
-      <c r="P17" s="5"/>
-      <c r="Q17" s="5"/>
-    </row>
-    <row r="18" spans="1:17" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="5"/>
-      <c r="B18" s="5"/>
-      <c r="C18" s="5"/>
-      <c r="D18" s="5"/>
-      <c r="E18" s="5"/>
-      <c r="F18" s="5"/>
-      <c r="G18" s="5"/>
-      <c r="H18" s="5"/>
-      <c r="I18" s="5"/>
-      <c r="J18" s="5"/>
-      <c r="K18" s="5"/>
-      <c r="L18" s="5"/>
-      <c r="M18" s="5"/>
-      <c r="N18" s="5"/>
-      <c r="O18" s="5"/>
-      <c r="P18" s="5"/>
-      <c r="Q18" s="5"/>
-    </row>
-    <row r="19" spans="1:17" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="5"/>
-      <c r="B19" s="5"/>
-      <c r="C19" s="5"/>
-      <c r="D19" s="5"/>
-      <c r="E19" s="5"/>
-      <c r="F19" s="5"/>
-      <c r="G19" s="5"/>
-      <c r="H19" s="5"/>
-      <c r="I19" s="5"/>
-      <c r="J19" s="5"/>
-      <c r="K19" s="5"/>
-      <c r="L19" s="5"/>
-      <c r="M19" s="5"/>
-      <c r="N19" s="5"/>
-      <c r="O19" s="5"/>
-      <c r="P19" s="5"/>
-      <c r="Q19" s="5"/>
-    </row>
-    <row r="20" spans="1:17" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="5"/>
-      <c r="B20" s="5"/>
-      <c r="C20" s="5"/>
-      <c r="D20" s="5"/>
-      <c r="E20" s="5"/>
-      <c r="F20" s="5"/>
-      <c r="G20" s="5"/>
-      <c r="H20" s="5"/>
-      <c r="I20" s="5"/>
-      <c r="J20" s="5"/>
-      <c r="K20" s="5"/>
-      <c r="L20" s="5"/>
-      <c r="M20" s="5"/>
-      <c r="N20" s="5"/>
-      <c r="O20" s="5"/>
-      <c r="P20" s="5"/>
-      <c r="Q20" s="5"/>
-    </row>
-    <row r="21" spans="1:17" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="5"/>
-      <c r="B21" s="5"/>
-      <c r="C21" s="5"/>
-      <c r="D21" s="5"/>
-      <c r="E21" s="5"/>
-      <c r="F21" s="5"/>
-      <c r="G21" s="5"/>
-      <c r="H21" s="5"/>
-      <c r="I21" s="5"/>
-      <c r="J21" s="5"/>
-      <c r="K21" s="5"/>
-      <c r="L21" s="5"/>
-      <c r="M21" s="5"/>
-      <c r="N21" s="5"/>
-      <c r="O21" s="5"/>
-      <c r="P21" s="5"/>
-      <c r="Q21" s="5"/>
-    </row>
-    <row r="22" spans="1:17" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="5"/>
-      <c r="B22" s="5"/>
-      <c r="C22" s="5"/>
-      <c r="D22" s="5"/>
-      <c r="E22" s="5"/>
-      <c r="F22" s="5"/>
-      <c r="G22" s="5"/>
-      <c r="H22" s="5"/>
-      <c r="I22" s="5"/>
-      <c r="J22" s="5"/>
-      <c r="K22" s="5"/>
-      <c r="L22" s="5"/>
-      <c r="M22" s="5"/>
-      <c r="N22" s="5"/>
-      <c r="O22" s="5"/>
-      <c r="P22" s="5"/>
-      <c r="Q22" s="5"/>
-    </row>
-    <row r="23" spans="1:17" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="5"/>
-      <c r="B23" s="5"/>
-      <c r="C23" s="5"/>
-      <c r="D23" s="5"/>
-      <c r="E23" s="5"/>
-      <c r="F23" s="5"/>
-      <c r="G23" s="5"/>
-      <c r="H23" s="5"/>
-      <c r="I23" s="5"/>
-      <c r="J23" s="5"/>
-      <c r="K23" s="5"/>
-      <c r="L23" s="5"/>
-      <c r="M23" s="5"/>
-      <c r="N23" s="5"/>
-      <c r="O23" s="5"/>
-      <c r="P23" s="5"/>
-      <c r="Q23" s="5"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
@@ -1765,7 +1190,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5DDF0F5E-A868-4567-9975-60FD4D7C0086}">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
@@ -1778,7 +1203,7 @@
     <col min="3" max="3" width="16.5546875" style="9" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="35.6640625" style="9" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="13" style="9" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="37.33203125" style="9" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="17.88671875" style="9" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="24.33203125" style="9" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="17.33203125" style="9" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="21.33203125" style="9" bestFit="1" customWidth="1"/>
@@ -1790,7 +1215,7 @@
     <col min="15" max="16" width="8.6640625" style="9" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" s="9" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:16" s="9" customFormat="1" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1840,7 +1265,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:16" s="9" customFormat="1" ht="33" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:16" s="9" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A2" s="4">
         <v>1</v>
       </c>
@@ -1849,24 +1274,24 @@
       </c>
       <c r="C2" s="5"/>
       <c r="D2" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="E2" s="5"/>
+        <v>51</v>
+      </c>
+      <c r="E2" s="5" t="s">
+        <v>57</v>
+      </c>
       <c r="F2" s="5" t="s">
-        <v>18</v>
+        <v>54</v>
       </c>
       <c r="G2" s="5" t="s">
-        <v>19</v>
+        <v>61</v>
       </c>
       <c r="H2" s="5" t="s">
-        <v>20</v>
+        <v>60</v>
       </c>
       <c r="I2" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="J2" s="5" t="s">
-        <v>21</v>
-      </c>
+        <v>48</v>
+      </c>
+      <c r="J2" s="5"/>
       <c r="K2" s="5"/>
       <c r="L2" s="5"/>
       <c r="M2" s="5"/>
@@ -1874,7 +1299,7 @@
       <c r="O2" s="5"/>
       <c r="P2" s="5"/>
     </row>
-    <row r="3" spans="1:16" s="9" customFormat="1" ht="33" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:16" s="9" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A3" s="4">
         <v>2</v>
       </c>
@@ -1883,24 +1308,24 @@
       </c>
       <c r="C3" s="5"/>
       <c r="D3" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="E3" s="5"/>
+        <v>49</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>58</v>
+      </c>
       <c r="F3" s="5" t="s">
-        <v>23</v>
+        <v>55</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>19</v>
+        <v>50</v>
       </c>
       <c r="H3" s="5" t="s">
-        <v>20</v>
+        <v>60</v>
       </c>
       <c r="I3" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="J3" s="5" t="s">
-        <v>25</v>
-      </c>
+        <v>48</v>
+      </c>
+      <c r="J3" s="5"/>
       <c r="K3" s="5"/>
       <c r="L3" s="5"/>
       <c r="M3" s="5"/>
@@ -1908,7 +1333,7 @@
       <c r="O3" s="5"/>
       <c r="P3" s="5"/>
     </row>
-    <row r="4" spans="1:16" s="9" customFormat="1" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:16" s="9" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A4" s="4">
         <v>3</v>
       </c>
@@ -1917,24 +1342,22 @@
       </c>
       <c r="C4" s="6"/>
       <c r="D4" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="E4" s="6"/>
+        <v>52</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>57</v>
+      </c>
       <c r="F4" s="5" t="s">
-        <v>27</v>
+        <v>56</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>19</v>
+        <v>53</v>
       </c>
       <c r="H4" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="I4" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="J4" s="5" t="s">
-        <v>21</v>
-      </c>
+        <v>60</v>
+      </c>
+      <c r="I4" s="5"/>
+      <c r="J4" s="5"/>
       <c r="K4" s="6"/>
       <c r="L4" s="6"/>
       <c r="M4" s="6"/>
@@ -1942,7 +1365,7 @@
       <c r="O4" s="6"/>
       <c r="P4" s="6"/>
     </row>
-    <row r="5" spans="1:16" s="9" customFormat="1" ht="33" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:16" s="9" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A5" s="4">
         <v>4</v>
       </c>
@@ -1951,24 +1374,18 @@
       </c>
       <c r="C5" s="5"/>
       <c r="D5" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="E5" s="5"/>
+        <v>59</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>58</v>
+      </c>
       <c r="F5" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="G5" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="H5" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="I5" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="J5" s="5" t="s">
-        <v>25</v>
-      </c>
+        <v>55</v>
+      </c>
+      <c r="G5" s="5"/>
+      <c r="H5" s="5"/>
+      <c r="I5" s="5"/>
+      <c r="J5" s="5"/>
       <c r="K5" s="5"/>
       <c r="L5" s="5"/>
       <c r="M5" s="5"/>
@@ -1976,7 +1393,7 @@
       <c r="O5" s="5"/>
       <c r="P5" s="5"/>
     </row>
-    <row r="6" spans="1:16" s="9" customFormat="1" ht="33" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:16" s="9" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A6" s="4">
         <v>5</v>
       </c>
@@ -1984,25 +1401,13 @@
         <v>28</v>
       </c>
       <c r="C6" s="5"/>
-      <c r="D6" s="5" t="s">
-        <v>33</v>
-      </c>
+      <c r="D6" s="5"/>
       <c r="E6" s="5"/>
-      <c r="F6" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="G6" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="H6" s="5" t="s">
-        <v>35</v>
-      </c>
-      <c r="I6" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="J6" s="5" t="s">
-        <v>25</v>
-      </c>
+      <c r="F6" s="5"/>
+      <c r="G6" s="5"/>
+      <c r="H6" s="5"/>
+      <c r="I6" s="5"/>
+      <c r="J6" s="5"/>
       <c r="K6" s="5"/>
       <c r="L6" s="5"/>
       <c r="M6" s="5"/>
@@ -2010,7 +1415,7 @@
       <c r="O6" s="5"/>
       <c r="P6" s="5"/>
     </row>
-    <row r="7" spans="1:16" s="9" customFormat="1" ht="33" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:16" s="9" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A7" s="4">
         <v>6</v>
       </c>
@@ -2018,25 +1423,13 @@
         <v>28</v>
       </c>
       <c r="C7" s="5"/>
-      <c r="D7" s="5" t="s">
-        <v>36</v>
-      </c>
+      <c r="D7" s="5"/>
       <c r="E7" s="5"/>
-      <c r="F7" s="5" t="s">
-        <v>37</v>
-      </c>
-      <c r="G7" s="5" t="s">
-        <v>38</v>
-      </c>
-      <c r="H7" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="I7" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="J7" s="5" t="s">
-        <v>25</v>
-      </c>
+      <c r="F7" s="5"/>
+      <c r="G7" s="5"/>
+      <c r="H7" s="5"/>
+      <c r="I7" s="5"/>
+      <c r="J7" s="5"/>
       <c r="K7" s="5"/>
       <c r="L7" s="5"/>
       <c r="M7" s="5"/>
@@ -2044,7 +1437,7 @@
       <c r="O7" s="5"/>
       <c r="P7" s="5"/>
     </row>
-    <row r="8" spans="1:16" s="9" customFormat="1" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:16" s="9" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A8" s="4">
         <v>7</v>
       </c>
@@ -2052,25 +1445,13 @@
         <v>28</v>
       </c>
       <c r="C8" s="5"/>
-      <c r="D8" s="5" t="s">
-        <v>39</v>
-      </c>
+      <c r="D8" s="5"/>
       <c r="E8" s="5"/>
-      <c r="F8" s="5" t="s">
-        <v>40</v>
-      </c>
-      <c r="G8" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="H8" s="5" t="s">
-        <v>41</v>
-      </c>
-      <c r="I8" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="J8" s="5" t="s">
-        <v>21</v>
-      </c>
+      <c r="F8" s="5"/>
+      <c r="G8" s="5"/>
+      <c r="H8" s="5"/>
+      <c r="I8" s="5"/>
+      <c r="J8" s="5"/>
       <c r="K8" s="5"/>
       <c r="L8" s="5"/>
       <c r="M8" s="5"/>
@@ -2078,7 +1459,7 @@
       <c r="O8" s="6"/>
       <c r="P8" s="6"/>
     </row>
-    <row r="9" spans="1:16" s="9" customFormat="1" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:16" s="9" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A9" s="4">
         <v>8</v>
       </c>
@@ -2086,25 +1467,13 @@
         <v>28</v>
       </c>
       <c r="C9" s="5"/>
-      <c r="D9" s="5" t="s">
-        <v>43</v>
-      </c>
+      <c r="D9" s="5"/>
       <c r="E9" s="5"/>
-      <c r="F9" s="5" t="s">
-        <v>44</v>
-      </c>
-      <c r="G9" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="H9" s="5" t="s">
-        <v>45</v>
-      </c>
-      <c r="I9" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="J9" s="5" t="s">
-        <v>25</v>
-      </c>
+      <c r="F9" s="5"/>
+      <c r="G9" s="5"/>
+      <c r="H9" s="5"/>
+      <c r="I9" s="5"/>
+      <c r="J9" s="5"/>
       <c r="K9" s="5"/>
       <c r="L9" s="5"/>
       <c r="M9" s="5"/>
@@ -2112,7 +1481,7 @@
       <c r="O9" s="6"/>
       <c r="P9" s="6"/>
     </row>
-    <row r="10" spans="1:16" s="9" customFormat="1" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:16" s="9" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A10" s="4">
         <v>9</v>
       </c>
@@ -2120,25 +1489,13 @@
         <v>28</v>
       </c>
       <c r="C10" s="5"/>
-      <c r="D10" s="5" t="s">
-        <v>46</v>
-      </c>
+      <c r="D10" s="5"/>
       <c r="E10" s="5"/>
-      <c r="F10" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="G10" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="H10" s="5" t="s">
-        <v>45</v>
-      </c>
-      <c r="I10" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="J10" s="5" t="s">
-        <v>25</v>
-      </c>
+      <c r="F10" s="5"/>
+      <c r="G10" s="5"/>
+      <c r="H10" s="5"/>
+      <c r="I10" s="5"/>
+      <c r="J10" s="5"/>
       <c r="K10" s="5"/>
       <c r="L10" s="5"/>
       <c r="M10" s="5"/>
@@ -2329,13 +1686,4 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{55AAD7F6-DF92-44C8-BC9F-081C8DAED1DE}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Add search functionality tests for hotel and flight
</commit_message>
<xml_diff>
--- a/TestCase_Integration_login.xlsx
+++ b/TestCase_Integration_login.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Desktop\travel_auto_test\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2DF6685-BBD8-49D9-9E68-B32101252804}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EAA81866-673F-4237-B9DE-D1E0254A387B}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="480" yWindow="60" windowWidth="18192" windowHeight="8508" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="480" yWindow="60" windowWidth="18192" windowHeight="8508" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="login" sheetId="2" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="187" uniqueCount="91">
   <si>
     <t>Test Case ID</t>
   </si>
@@ -179,21 +179,6 @@
     <t>A trip to New York shows up</t>
   </si>
   <si>
-    <t>Search flight</t>
-  </si>
-  <si>
-    <t>navigate to services, enter flight</t>
-  </si>
-  <si>
-    <t>Search hotel</t>
-  </si>
-  <si>
-    <t>Search hotel but uppercase destination</t>
-  </si>
-  <si>
-    <t>navigate to services, enter hotel</t>
-  </si>
-  <si>
     <t>hotel = "New york"
 Flight = ""</t>
   </si>
@@ -209,16 +194,130 @@
     <t>at least one hotel named New York</t>
   </si>
   <si>
-    <t>at least one flight named A380</t>
-  </si>
-  <si>
-    <t>Search flight but lowercase flight</t>
-  </si>
-  <si>
     <t>Found a trip to New York</t>
   </si>
   <si>
     <t>navigate to services, enter hotel name, press button search</t>
+  </si>
+  <si>
+    <t>hotel = ""
+Flight = "a380"</t>
+  </si>
+  <si>
+    <t>Search hotel in New York and flight in New York</t>
+  </si>
+  <si>
+    <t>hotel = "New york"
+Flight = "Flight A380"</t>
+  </si>
+  <si>
+    <t>Search hotel in Paris and flight in New York</t>
+  </si>
+  <si>
+    <t>Two trips, one to Paris, one to New York</t>
+  </si>
+  <si>
+    <t>hotel = "Paris"
+Flight = "Flight B787"</t>
+  </si>
+  <si>
+    <t>navigate to services, enter flight, press button search</t>
+  </si>
+  <si>
+    <t>navigate to services, enter hotel and flight, press button search</t>
+  </si>
+  <si>
+    <t>No trip is found</t>
+  </si>
+  <si>
+    <t>Search partial flight name</t>
+  </si>
+  <si>
+    <t>hotel = ""
+Flight = "A3"</t>
+  </si>
+  <si>
+    <t>Search partial hotel name</t>
+  </si>
+  <si>
+    <t>hotel = "New"
+Flight = ""</t>
+  </si>
+  <si>
+    <t>Search hotel with trailing space</t>
+  </si>
+  <si>
+    <t>Search flight with trailing space</t>
+  </si>
+  <si>
+    <t>hotel = "    New york    "
+Flight = ""</t>
+  </si>
+  <si>
+    <t>hotel = ""
+Flight = "    A380   "</t>
+  </si>
+  <si>
+    <t>A trip to New York has flight and hotel</t>
+  </si>
+  <si>
+    <t>Search exact hotel</t>
+  </si>
+  <si>
+    <t>Search exact flight</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Search hotel but uppercase </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Search flight but lowercase </t>
+  </si>
+  <si>
+    <t>Search hotel but mixed case</t>
+  </si>
+  <si>
+    <t>hotel = "NeW yOrk"
+Flight = ""</t>
+  </si>
+  <si>
+    <t>Search no space hotel</t>
+  </si>
+  <si>
+    <t>hotel = "Newyork"
+Flight = ""</t>
+  </si>
+  <si>
+    <t>Search hotel and flight are both empty</t>
+  </si>
+  <si>
+    <t>navigate to services, press button search</t>
+  </si>
+  <si>
+    <t>hotel = ""
+Flight = ""</t>
+  </si>
+  <si>
+    <t>Found all trips</t>
+  </si>
+  <si>
+    <t>There are trips are in database</t>
+  </si>
+  <si>
+    <t>Search nonexistent hotel</t>
+  </si>
+  <si>
+    <t>hotel = "hanoi"
+Flight = ""</t>
+  </si>
+  <si>
+    <t>Search nonexistent flight</t>
+  </si>
+  <si>
+    <t>hotel = ""
+Flight = "MH370"</t>
+  </si>
+  <si>
+    <t>navigate to services, enter flight name, press button search</t>
   </si>
 </sst>
 </file>
@@ -1195,23 +1294,23 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:P20"/>
+  <dimension ref="A1:P19"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="11" style="8" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="20.6640625" style="9" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="16.5546875" style="9" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="35.6640625" style="9" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13" style="9" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="17.88671875" style="9" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="24.33203125" style="9" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="17.33203125" style="9" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="21.33203125" style="9" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="6.33203125" style="9" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.21875" style="9" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="33.109375" style="9" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="26.109375" style="9" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="20.21875" style="9" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="44.44140625" style="9" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="21.5546875" style="9" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="16" style="9" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="6.21875" style="9" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="7.109375" style="9" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="7.6640625" style="9" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="6.77734375" style="9" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="6.109375" style="9" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="7.109375" style="9" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="5.33203125" style="9" bestFit="1" customWidth="1"/>
     <col min="15" max="16" width="8.6640625" style="9" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1265,7 +1364,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:16" s="9" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:16" s="9" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A2" s="4">
         <v>1</v>
       </c>
@@ -1274,19 +1373,19 @@
       </c>
       <c r="C2" s="5"/>
       <c r="D2" s="5" t="s">
-        <v>51</v>
+        <v>73</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="F2" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="G2" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="G2" s="5" t="s">
-        <v>61</v>
-      </c>
       <c r="H2" s="5" t="s">
-        <v>60</v>
+        <v>53</v>
       </c>
       <c r="I2" s="5" t="s">
         <v>48</v>
@@ -1299,7 +1398,7 @@
       <c r="O2" s="5"/>
       <c r="P2" s="5"/>
     </row>
-    <row r="3" spans="1:16" s="9" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:16" s="9" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A3" s="4">
         <v>2</v>
       </c>
@@ -1308,19 +1407,19 @@
       </c>
       <c r="C3" s="5"/>
       <c r="D3" s="5" t="s">
-        <v>49</v>
+        <v>74</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>58</v>
+        <v>72</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>50</v>
+        <v>61</v>
       </c>
       <c r="H3" s="5" t="s">
-        <v>60</v>
+        <v>53</v>
       </c>
       <c r="I3" s="5" t="s">
         <v>48</v>
@@ -1333,7 +1432,7 @@
       <c r="O3" s="5"/>
       <c r="P3" s="5"/>
     </row>
-    <row r="4" spans="1:16" s="9" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:16" s="9" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A4" s="4">
         <v>3</v>
       </c>
@@ -1342,19 +1441,19 @@
       </c>
       <c r="C4" s="6"/>
       <c r="D4" s="5" t="s">
-        <v>52</v>
+        <v>75</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>57</v>
+        <v>72</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="G4" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="H4" s="5" t="s">
         <v>53</v>
-      </c>
-      <c r="H4" s="5" t="s">
-        <v>60</v>
       </c>
       <c r="I4" s="5"/>
       <c r="J4" s="5"/>
@@ -1365,25 +1464,29 @@
       <c r="O4" s="6"/>
       <c r="P4" s="6"/>
     </row>
-    <row r="5" spans="1:16" s="9" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:16" s="9" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A5" s="4">
         <v>4</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>28</v>
+        <v>16</v>
       </c>
       <c r="C5" s="5"/>
       <c r="D5" s="5" t="s">
-        <v>59</v>
+        <v>76</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>58</v>
+        <v>72</v>
       </c>
       <c r="F5" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="G5" s="5"/>
-      <c r="H5" s="5"/>
+      <c r="G5" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="H5" s="5" t="s">
+        <v>53</v>
+      </c>
       <c r="I5" s="5"/>
       <c r="J5" s="5"/>
       <c r="K5" s="5"/>
@@ -1393,19 +1496,29 @@
       <c r="O5" s="5"/>
       <c r="P5" s="5"/>
     </row>
-    <row r="6" spans="1:16" s="9" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:16" s="9" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A6" s="4">
         <v>5</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>28</v>
+        <v>16</v>
       </c>
       <c r="C6" s="5"/>
-      <c r="D6" s="5"/>
-      <c r="E6" s="5"/>
-      <c r="F6" s="5"/>
-      <c r="G6" s="5"/>
-      <c r="H6" s="5"/>
+      <c r="D6" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="G6" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="H6" s="5" t="s">
+        <v>53</v>
+      </c>
       <c r="I6" s="5"/>
       <c r="J6" s="5"/>
       <c r="K6" s="5"/>
@@ -1415,7 +1528,7 @@
       <c r="O6" s="5"/>
       <c r="P6" s="5"/>
     </row>
-    <row r="7" spans="1:16" s="9" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:16" s="9" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A7" s="4">
         <v>6</v>
       </c>
@@ -1423,11 +1536,21 @@
         <v>28</v>
       </c>
       <c r="C7" s="5"/>
-      <c r="D7" s="5"/>
-      <c r="E7" s="5"/>
-      <c r="F7" s="5"/>
-      <c r="G7" s="5"/>
-      <c r="H7" s="5"/>
+      <c r="D7" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="F7" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="G7" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="H7" s="5" t="s">
+        <v>63</v>
+      </c>
       <c r="I7" s="5"/>
       <c r="J7" s="5"/>
       <c r="K7" s="5"/>
@@ -1437,19 +1560,29 @@
       <c r="O7" s="5"/>
       <c r="P7" s="5"/>
     </row>
-    <row r="8" spans="1:16" s="9" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:16" s="9" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A8" s="4">
         <v>7</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>28</v>
+        <v>16</v>
       </c>
       <c r="C8" s="5"/>
-      <c r="D8" s="5"/>
-      <c r="E8" s="5"/>
-      <c r="F8" s="5"/>
-      <c r="G8" s="5"/>
-      <c r="H8" s="5"/>
+      <c r="D8" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="E8" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="F8" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="G8" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="H8" s="5" t="s">
+        <v>53</v>
+      </c>
       <c r="I8" s="5"/>
       <c r="J8" s="5"/>
       <c r="K8" s="5"/>
@@ -1459,19 +1592,29 @@
       <c r="O8" s="6"/>
       <c r="P8" s="6"/>
     </row>
-    <row r="9" spans="1:16" s="9" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:16" s="9" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A9" s="4">
         <v>8</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>28</v>
+        <v>16</v>
       </c>
       <c r="C9" s="5"/>
-      <c r="D9" s="5"/>
-      <c r="E9" s="5"/>
-      <c r="F9" s="5"/>
-      <c r="G9" s="5"/>
-      <c r="H9" s="5"/>
+      <c r="D9" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="E9" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="F9" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="G9" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="H9" s="5" t="s">
+        <v>53</v>
+      </c>
       <c r="I9" s="5"/>
       <c r="J9" s="5"/>
       <c r="K9" s="5"/>
@@ -1481,19 +1624,29 @@
       <c r="O9" s="6"/>
       <c r="P9" s="6"/>
     </row>
-    <row r="10" spans="1:16" s="9" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:16" s="9" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A10" s="4">
         <v>9</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>28</v>
+        <v>16</v>
       </c>
       <c r="C10" s="5"/>
-      <c r="D10" s="5"/>
-      <c r="E10" s="5"/>
-      <c r="F10" s="5"/>
-      <c r="G10" s="5"/>
-      <c r="H10" s="5"/>
+      <c r="D10" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="E10" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="F10" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="G10" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="H10" s="5" t="s">
+        <v>53</v>
+      </c>
       <c r="I10" s="5"/>
       <c r="J10" s="5"/>
       <c r="K10" s="5"/>
@@ -1503,15 +1656,29 @@
       <c r="O10" s="6"/>
       <c r="P10" s="6"/>
     </row>
-    <row r="11" spans="1:16" s="9" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="7"/>
-      <c r="B11" s="6"/>
+    <row r="11" spans="1:16" s="9" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A11" s="4">
+        <v>10</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>16</v>
+      </c>
       <c r="C11" s="6"/>
-      <c r="D11" s="6"/>
-      <c r="E11" s="6"/>
-      <c r="F11" s="6"/>
-      <c r="G11" s="6"/>
-      <c r="H11" s="6"/>
+      <c r="D11" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="E11" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="F11" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="G11" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="H11" s="5" t="s">
+        <v>53</v>
+      </c>
       <c r="I11" s="6"/>
       <c r="J11" s="6"/>
       <c r="K11" s="6"/>
@@ -1521,15 +1688,29 @@
       <c r="O11" s="6"/>
       <c r="P11" s="6"/>
     </row>
-    <row r="12" spans="1:16" s="9" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="7"/>
-      <c r="B12" s="6"/>
+    <row r="12" spans="1:16" s="9" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A12" s="4">
+        <v>11</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>16</v>
+      </c>
       <c r="C12" s="6"/>
-      <c r="D12" s="6"/>
-      <c r="E12" s="6"/>
-      <c r="F12" s="6"/>
-      <c r="G12" s="6"/>
-      <c r="H12" s="6"/>
+      <c r="D12" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="E12" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="F12" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="G12" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="H12" s="5" t="s">
+        <v>53</v>
+      </c>
       <c r="I12" s="6"/>
       <c r="J12" s="6"/>
       <c r="K12" s="6"/>
@@ -1539,15 +1720,29 @@
       <c r="O12" s="6"/>
       <c r="P12" s="6"/>
     </row>
-    <row r="13" spans="1:16" s="9" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="7"/>
-      <c r="B13" s="6"/>
+    <row r="13" spans="1:16" s="9" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A13" s="4">
+        <v>12</v>
+      </c>
+      <c r="B13" s="5" t="s">
+        <v>16</v>
+      </c>
       <c r="C13" s="6"/>
-      <c r="D13" s="6"/>
-      <c r="E13" s="6"/>
-      <c r="F13" s="6"/>
-      <c r="G13" s="6"/>
-      <c r="H13" s="6"/>
+      <c r="D13" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="E13" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="F13" s="5" t="s">
+        <v>80</v>
+      </c>
+      <c r="G13" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="H13" s="5" t="s">
+        <v>53</v>
+      </c>
       <c r="I13" s="6"/>
       <c r="J13" s="6"/>
       <c r="K13" s="6"/>
@@ -1557,15 +1752,29 @@
       <c r="O13" s="6"/>
       <c r="P13" s="6"/>
     </row>
-    <row r="14" spans="1:16" s="9" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="7"/>
-      <c r="B14" s="6"/>
+    <row r="14" spans="1:16" s="9" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A14" s="4">
+        <v>13</v>
+      </c>
+      <c r="B14" s="6" t="s">
+        <v>16</v>
+      </c>
       <c r="C14" s="6"/>
-      <c r="D14" s="6"/>
-      <c r="E14" s="6"/>
-      <c r="F14" s="6"/>
-      <c r="G14" s="6"/>
-      <c r="H14" s="6"/>
+      <c r="D14" s="6" t="s">
+        <v>81</v>
+      </c>
+      <c r="E14" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="F14" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="G14" s="5" t="s">
+        <v>82</v>
+      </c>
+      <c r="H14" s="5" t="s">
+        <v>84</v>
+      </c>
       <c r="I14" s="6"/>
       <c r="J14" s="6"/>
       <c r="K14" s="6"/>
@@ -1575,15 +1784,29 @@
       <c r="O14" s="6"/>
       <c r="P14" s="6"/>
     </row>
-    <row r="15" spans="1:16" s="9" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="7"/>
-      <c r="B15" s="6"/>
+    <row r="15" spans="1:16" s="9" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A15" s="4">
+        <v>14</v>
+      </c>
+      <c r="B15" s="6" t="s">
+        <v>28</v>
+      </c>
       <c r="C15" s="6"/>
-      <c r="D15" s="6"/>
-      <c r="E15" s="6"/>
-      <c r="F15" s="6"/>
-      <c r="G15" s="6"/>
-      <c r="H15" s="6"/>
+      <c r="D15" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="E15" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="F15" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="G15" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="H15" s="5" t="s">
+        <v>63</v>
+      </c>
       <c r="I15" s="6"/>
       <c r="J15" s="6"/>
       <c r="K15" s="6"/>
@@ -1593,15 +1816,29 @@
       <c r="O15" s="6"/>
       <c r="P15" s="6"/>
     </row>
-    <row r="16" spans="1:16" s="9" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="7"/>
-      <c r="B16" s="6"/>
+    <row r="16" spans="1:16" s="9" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A16" s="4">
+        <v>15</v>
+      </c>
+      <c r="B16" s="6" t="s">
+        <v>28</v>
+      </c>
       <c r="C16" s="6"/>
-      <c r="D16" s="6"/>
-      <c r="E16" s="6"/>
-      <c r="F16" s="6"/>
-      <c r="G16" s="6"/>
-      <c r="H16" s="6"/>
+      <c r="D16" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="E16" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="F16" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="G16" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="H16" s="5" t="s">
+        <v>63</v>
+      </c>
       <c r="I16" s="6"/>
       <c r="J16" s="6"/>
       <c r="K16" s="6"/>
@@ -1647,7 +1884,7 @@
       <c r="O18" s="6"/>
       <c r="P18" s="6"/>
     </row>
-    <row r="19" spans="1:16" s="9" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:16" s="9" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="7"/>
       <c r="B19" s="6"/>
       <c r="C19" s="6"/>
@@ -1665,24 +1902,6 @@
       <c r="O19" s="6"/>
       <c r="P19" s="6"/>
     </row>
-    <row r="20" spans="1:16" s="9" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="7"/>
-      <c r="B20" s="6"/>
-      <c r="C20" s="6"/>
-      <c r="D20" s="6"/>
-      <c r="E20" s="6"/>
-      <c r="F20" s="6"/>
-      <c r="G20" s="6"/>
-      <c r="H20" s="6"/>
-      <c r="I20" s="6"/>
-      <c r="J20" s="6"/>
-      <c r="K20" s="6"/>
-      <c r="L20" s="6"/>
-      <c r="M20" s="6"/>
-      <c r="N20" s="6"/>
-      <c r="O20" s="6"/>
-      <c r="P20" s="6"/>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>